<commit_message>
Quick Update 2026-04-11 10:33
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -1,39 +1,456 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4275" yWindow="4005" windowWidth="38700" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet name="index" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="index" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <name val="Calibri"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="1">
+  <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="82.140625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="7.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="34.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="39.85546875" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="10.42578125" bestFit="1" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -324,5 +741,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Quick Update 2026-04-11 10:41
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -740,6 +740,38 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>cs_phone_battery_simulation</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>simulation</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>simulation;arrays</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Phone Battery Simulation</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>codesignal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Quick Update 2026-04-11 12:44
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -811,6 +811,38 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>lc_0084</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Largest Rectangle in Histogram</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Quick Update 2026-04-11 12:56
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -843,6 +843,38 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>lc_0150</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>stack;array;math</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Evaluate Reverse Polish Notation</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Quick Update 2026-04-11 14:19
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -875,6 +875,38 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>lc_0155</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>stack;design</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Min Stack</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Quick Update 2026-04-11 18:54
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -814,12 +814,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -846,12 +846,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -861,12 +861,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -878,30 +878,126 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>lc_0150</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>stack;array;math</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Evaluate Reverse Polish Notation</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>lc_0239</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Sliding Window Maximum</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>lc_0496</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Next Greater Element I</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-11 21:08
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -846,12 +846,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -878,12 +878,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -910,12 +910,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -925,12 +925,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -942,12 +942,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -974,30 +974,190 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>lc_0150</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>stack;array;math</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Evaluate Reverse Polish Notation</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>lc_0239</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Sliding Window Maximum</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>lc_0496</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Next Greater Element I</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>lc_0503</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Next Greater Element II</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-11 21:19
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -622,44 +622,44 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cs_drone_delivery_foot_distance</t>
+          <t>lc_0001</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
+          <t>leetcode/by_topic/arrays_hashing/001_lc_0001_two_sum_empty.py</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>greedy</t>
+          <t>arrays_hashing</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>greedy;simulation;sorting</t>
+          <t>arrays_hashing;arrays;hash-table</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Drone Delivery Foot Distance</t>
+          <t>Two Sum</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cs_key_changes_counter</t>
+          <t>cs_drone_delivery_foot_distance</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
+          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -669,12 +669,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>greedy;simulation;arrays;strings</t>
+          <t>greedy;simulation;sorting</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Key Changes Counter</t>
+          <t>Drone Delivery Foot Distance</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -686,12 +686,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings</t>
+          <t>cs_key_changes_counter</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
+          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -701,12 +701,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>greedy;math;array;sequence</t>
+          <t>greedy;simulation;arrays;strings</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns</t>
+          <t>Key Changes Counter</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -718,12 +718,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings_flexible</t>
+          <t>lc_custom_harmonious_buildings</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
+          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -733,12 +733,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>greedy;math;median;geometry</t>
+          <t>greedy;math;array;sequence</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns (Flexible)</t>
+          <t>Harmonious Building Patterns</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -750,27 +750,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_custom_harmonious_buildings_flexible</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>greedy</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>greedy;math;median;geometry</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Harmonious Building Patterns (Flexible)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -782,44 +782,44 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -829,12 +829,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -846,12 +846,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -878,12 +878,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -910,12 +910,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -925,12 +925,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -942,12 +942,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -974,12 +974,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -989,12 +989,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1006,12 +1006,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1021,12 +1021,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1038,12 +1038,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1053,12 +1053,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1070,12 +1070,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1102,12 +1102,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0503</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1117,12 +1117,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element II</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1134,30 +1134,62 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-11 22:02
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -654,76 +654,76 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cs_drone_delivery_foot_distance</t>
+          <t>lc_0036</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
+          <t>leetcode/by_topic/arrays_hashing/036_lc_036_valid_sudoku_empty.py</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>greedy</t>
+          <t>arrays_hashing</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>greedy;simulation;sorting</t>
+          <t>arrays_hashing;hash-table;matrix;set</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Drone Delivery Foot Distance</t>
+          <t>Valid Sudoku</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cs_key_changes_counter</t>
+          <t>lc_0049</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
+          <t>leetcode/by_topic/arrays_hashing/049_lc_049_group_anagrams_empty.py</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>greedy</t>
+          <t>arrays_hashing</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>greedy;simulation;arrays;strings</t>
+          <t>arrays_hashing;hash-table;strings;sorting</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Key Changes Counter</t>
+          <t>Group Anagrams</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings</t>
+          <t>cs_drone_delivery_foot_distance</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
+          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -733,12 +733,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>greedy;math;array;sequence</t>
+          <t>greedy;simulation;sorting</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns</t>
+          <t>Drone Delivery Foot Distance</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -750,12 +750,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings_flexible</t>
+          <t>cs_key_changes_counter</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
+          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -765,12 +765,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>greedy;math;median;geometry</t>
+          <t>greedy;simulation;arrays;strings</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns (Flexible)</t>
+          <t>Key Changes Counter</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -782,27 +782,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_custom_harmonious_buildings</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>greedy</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>greedy;math;array;sequence</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Harmonious Building Patterns</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -814,76 +814,76 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>lc_custom_harmonious_buildings_flexible</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>greedy</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>greedy;math;median;geometry</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Harmonious Building Patterns (Flexible)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -910,12 +910,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -930,7 +930,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -942,12 +942,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -974,12 +974,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -989,12 +989,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1006,12 +1006,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1021,12 +1021,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1038,12 +1038,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1053,12 +1053,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1070,12 +1070,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1102,12 +1102,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1117,12 +1117,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1134,12 +1134,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1166,30 +1166,94 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>lc_0503</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Next Greater Element II</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-11 22:08
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -718,44 +718,44 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cs_drone_delivery_foot_distance</t>
+          <t>lc_0128</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
+          <t>leetcode/by_topic/arrays_hashing/128_lc_128_longest_consecutive_sequence_empty.py</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>greedy</t>
+          <t>arrays_hashing</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>greedy;simulation;sorting</t>
+          <t>arrays_hashing;hash-table;arrays;union-find</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Drone Delivery Foot Distance</t>
+          <t>Longest Consecutive Sequence</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cs_key_changes_counter</t>
+          <t>cs_drone_delivery_foot_distance</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
+          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -765,12 +765,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>greedy;simulation;arrays;strings</t>
+          <t>greedy;simulation;sorting</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Key Changes Counter</t>
+          <t>Drone Delivery Foot Distance</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -782,12 +782,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings</t>
+          <t>cs_key_changes_counter</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
+          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -797,12 +797,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>greedy;math;array;sequence</t>
+          <t>greedy;simulation;arrays;strings</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns</t>
+          <t>Key Changes Counter</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings_flexible</t>
+          <t>lc_custom_harmonious_buildings</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
+          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -829,12 +829,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>greedy;math;median;geometry</t>
+          <t>greedy;math;array;sequence</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns (Flexible)</t>
+          <t>Harmonious Building Patterns</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -846,27 +846,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_custom_harmonious_buildings_flexible</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>greedy</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>greedy;math;median;geometry</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Harmonious Building Patterns (Flexible)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -878,44 +878,44 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -925,12 +925,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -942,12 +942,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -974,12 +974,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1006,12 +1006,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1021,12 +1021,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1038,12 +1038,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1053,12 +1053,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1070,12 +1070,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1102,12 +1102,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1117,12 +1117,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1134,12 +1134,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1166,12 +1166,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1181,12 +1181,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1198,12 +1198,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0503</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element II</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1230,30 +1230,62 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-11 22:20
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -750,76 +750,76 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cs_drone_delivery_foot_distance</t>
+          <t>lc_0217</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
+          <t>leetcode/by_topic/arrays_hashing/217_lc_0217_contains_duplicate_empty.py</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>greedy</t>
+          <t>arrays_hashing</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>greedy;simulation;sorting</t>
+          <t>arrays_hashing;hash-table;arrays;sorting</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Drone Delivery Foot Distance</t>
+          <t>Contains Duplicate</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cs_key_changes_counter</t>
+          <t>lc_0242</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
+          <t>leetcode/by_topic/arrays_hashing/242_lc_0242_valid_anagram_empty.py</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>greedy</t>
+          <t>arrays_hashing</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>greedy;simulation;arrays;strings</t>
+          <t>arrays_hashing;hash-table;strings;sorting</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Key Changes Counter</t>
+          <t>Valid Anagram</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings</t>
+          <t>cs_drone_delivery_foot_distance</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
+          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -829,12 +829,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>greedy;math;array;sequence</t>
+          <t>greedy;simulation;sorting</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns</t>
+          <t>Drone Delivery Foot Distance</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -846,12 +846,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings_flexible</t>
+          <t>cs_key_changes_counter</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
+          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -861,12 +861,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>greedy;math;median;geometry</t>
+          <t>greedy;simulation;arrays;strings</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns (Flexible)</t>
+          <t>Key Changes Counter</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -878,27 +878,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_custom_harmonious_buildings</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>greedy</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>greedy;math;array;sequence</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Harmonious Building Patterns</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -910,76 +910,76 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>lc_custom_harmonious_buildings_flexible</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>greedy</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>greedy;math;median;geometry</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Harmonious Building Patterns (Flexible)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -989,12 +989,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1006,12 +1006,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1038,12 +1038,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1053,12 +1053,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1070,12 +1070,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1102,12 +1102,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1117,12 +1117,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1134,12 +1134,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1166,12 +1166,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1181,12 +1181,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1198,12 +1198,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1230,12 +1230,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1245,12 +1245,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1262,30 +1262,94 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>lc_0503</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Next Greater Element II</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-11 23:53
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -814,44 +814,44 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>cs_drone_delivery_foot_distance</t>
+          <t>lc_0271</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
+          <t>leetcode/by_topic/arrays_hashing/271_lc_0271_encode_and_decode_strings_empty.py</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>greedy</t>
+          <t>arrays_hashing</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>greedy;simulation;sorting</t>
+          <t>arrays_hashing;strings;design;encoding</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Drone Delivery Foot Distance</t>
+          <t>Encode and Decode Strings</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cs_key_changes_counter</t>
+          <t>cs_drone_delivery_foot_distance</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
+          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -861,12 +861,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>greedy;simulation;arrays;strings</t>
+          <t>greedy;simulation;sorting</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Key Changes Counter</t>
+          <t>Drone Delivery Foot Distance</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -878,12 +878,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings</t>
+          <t>cs_key_changes_counter</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
+          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>greedy;math;array;sequence</t>
+          <t>greedy;simulation;arrays;strings</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns</t>
+          <t>Key Changes Counter</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -910,12 +910,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings_flexible</t>
+          <t>lc_custom_harmonious_buildings</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
+          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -925,12 +925,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>greedy;math;median;geometry</t>
+          <t>greedy;math;array;sequence</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns (Flexible)</t>
+          <t>Harmonious Building Patterns</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -942,27 +942,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_custom_harmonious_buildings_flexible</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>greedy</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>greedy;math;median;geometry</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Harmonious Building Patterns (Flexible)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -974,44 +974,44 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1021,12 +1021,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1038,12 +1038,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1070,12 +1070,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1102,12 +1102,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1117,12 +1117,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1134,12 +1134,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1166,12 +1166,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1181,12 +1181,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1198,12 +1198,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1230,12 +1230,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1245,12 +1245,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1262,12 +1262,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1277,12 +1277,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1294,12 +1294,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0503</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element II</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1326,30 +1326,62 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 00:26
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -846,76 +846,76 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cs_drone_delivery_foot_distance</t>
+          <t>lc_0347</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
+          <t>leetcode/by_topic/arrays_hashing/347_lc_0347_top_k_frequent_elements_empty.py</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>greedy</t>
+          <t>arrays_hashing</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>greedy;simulation;sorting</t>
+          <t>arrays_hashing;hash-table;heap;bucket-sort;counting</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Drone Delivery Foot Distance</t>
+          <t>Top K Frequent Elements</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cs_key_changes_counter</t>
+          <t>lc_0560</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
+          <t>leetcode/by_topic/arrays_hashing/560_lc_0560_subarray_sum_equals_k_empty.py</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>greedy</t>
+          <t>arrays_hashing</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>greedy;simulation;arrays;strings</t>
+          <t>arrays_hashing;hash-table;prefix-sum;arrays</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Key Changes Counter</t>
+          <t>Subarray Sum Equals K</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings</t>
+          <t>cs_drone_delivery_foot_distance</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
+          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -925,12 +925,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>greedy;math;array;sequence</t>
+          <t>greedy;simulation;sorting</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns</t>
+          <t>Drone Delivery Foot Distance</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -942,12 +942,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings_flexible</t>
+          <t>cs_key_changes_counter</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
+          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>greedy;math;median;geometry</t>
+          <t>greedy;simulation;arrays;strings</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns (Flexible)</t>
+          <t>Key Changes Counter</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -974,27 +974,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_custom_harmonious_buildings</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>greedy</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>greedy;math;array;sequence</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Harmonious Building Patterns</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1006,76 +1006,76 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>lc_custom_harmonious_buildings_flexible</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>greedy</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>greedy;math;median;geometry</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Harmonious Building Patterns (Flexible)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1102,12 +1102,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1134,12 +1134,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1166,12 +1166,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1181,12 +1181,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1198,12 +1198,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1230,12 +1230,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1245,12 +1245,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1262,12 +1262,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1277,12 +1277,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1294,12 +1294,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1326,12 +1326,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1341,12 +1341,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1358,30 +1358,94 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>lc_0503</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Next Greater Element II</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 01:45
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1038,59 +1038,59 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_1019</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>monotonic_stack</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Next Greater Node In Linked List</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>lc_1475</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>monotonic_stack</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Final Prices With a Special Discount in a Shop</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1102,44 +1102,44 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1166,12 +1166,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1198,12 +1198,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1230,12 +1230,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1245,12 +1245,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1262,12 +1262,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1277,12 +1277,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1294,12 +1294,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1326,12 +1326,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1341,12 +1341,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1358,12 +1358,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1373,12 +1373,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1390,12 +1390,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1405,12 +1405,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1422,30 +1422,94 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>lc_0503</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Next Greater Element II</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 01:48
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4275" yWindow="4005" windowWidth="38700" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1620" yWindow="5250" windowWidth="38700" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="index" sheetId="1" state="visible" r:id="rId1"/>
@@ -448,11 +448,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="82.140625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="89.5703125" bestFit="1" customWidth="1" min="2" max="2"/>
     <col width="17.85546875" customWidth="1" min="3" max="3"/>
     <col width="41.28515625" customWidth="1" min="4" max="4"/>
     <col width="39.85546875" bestFit="1" customWidth="1" min="5" max="5"/>
@@ -1038,12 +1038,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>lc_1019</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/084_lc_084_largest_rectangle_in_histogram_empty.py</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1053,12 +1053,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Next Greater Node In Linked List</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1070,12 +1070,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>lc_1475</t>
+          <t>lc_1019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Final Prices With a Special Discount in a Shop</t>
+          <t>Next Greater Node In Linked List</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1102,76 +1102,76 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_1475</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>monotonic_stack</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Final Prices With a Special Discount in a Shop</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1181,12 +1181,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1198,12 +1198,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1230,12 +1230,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1262,12 +1262,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1277,12 +1277,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1294,12 +1294,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1326,12 +1326,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1341,12 +1341,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1358,12 +1358,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1373,12 +1373,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1390,12 +1390,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1405,12 +1405,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1422,12 +1422,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1437,12 +1437,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1454,12 +1454,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0503</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element II</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1486,30 +1486,62 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 10:47
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1070,12 +1070,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>lc_1019</t>
+          <t>lc_0085</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/085_lc_085_maximal_rectangle_empty.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;dynamic-programming;matrix</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Next Greater Node In Linked List</t>
+          <t>Maximal Rectangle</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1102,12 +1102,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lc_1475</t>
+          <t>lc_1019</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1117,12 +1117,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Final Prices With a Special Discount in a Shop</t>
+          <t>Next Greater Node In Linked List</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1134,76 +1134,76 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_1475</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>monotonic_stack</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Final Prices With a Special Discount in a Shop</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1230,12 +1230,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1262,12 +1262,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1294,12 +1294,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1326,12 +1326,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1341,12 +1341,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1358,12 +1358,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1373,12 +1373,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1390,12 +1390,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1405,12 +1405,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1422,12 +1422,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1437,12 +1437,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1454,12 +1454,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1486,12 +1486,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0503</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1501,12 +1501,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element II</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1518,30 +1518,62 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 10:58
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1038,12 +1038,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0042</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/084_lc_084_largest_rectangle_in_histogram_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/042_lc_042_trapping_rain_water_empty.py</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1053,12 +1053,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;two-pointers;dynamic-programming</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Trapping Rain Water</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1070,12 +1070,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>lc_0085</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/085_lc_085_maximal_rectangle_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/084_lc_084_largest_rectangle_in_histogram_empty.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;dynamic-programming;matrix</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Maximal Rectangle</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1102,12 +1102,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lc_1019</t>
+          <t>lc_0085</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/085_lc_085_maximal_rectangle_empty.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1117,12 +1117,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;dynamic-programming;matrix</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Next Greater Node In Linked List</t>
+          <t>Maximal Rectangle</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1134,12 +1134,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>lc_1475</t>
+          <t>lc_1019</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Final Prices With a Special Discount in a Shop</t>
+          <t>Next Greater Node In Linked List</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1166,76 +1166,76 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_1475</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>monotonic_stack</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Final Prices With a Special Discount in a Shop</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1245,12 +1245,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1262,12 +1262,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1294,12 +1294,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1326,12 +1326,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1341,12 +1341,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1358,12 +1358,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1373,12 +1373,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1390,12 +1390,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1405,12 +1405,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1422,12 +1422,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1437,12 +1437,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1454,12 +1454,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1486,12 +1486,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1501,12 +1501,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1518,12 +1518,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0503</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1533,12 +1533,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element II</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1550,30 +1550,62 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 11:10
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1198,76 +1198,76 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>907_lc_0907_sum_of_subarray_minimums_empty</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/monotonic_stack/907_lc_0907_sum_of_subarray_minimums_empty.py</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>monotonic_stack</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>monotonic_stack</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>907 Lc 0907 Sum Of Subarray Minimums Empty</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1277,12 +1277,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1294,12 +1294,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1326,12 +1326,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1358,12 +1358,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1373,12 +1373,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1390,12 +1390,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1405,12 +1405,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1422,12 +1422,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1437,12 +1437,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1454,12 +1454,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1486,12 +1486,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1501,12 +1501,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1518,12 +1518,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1533,12 +1533,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1550,12 +1550,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0503</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1565,12 +1565,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element II</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1582,30 +1582,62 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 11:51
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -1198,7 +1198,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>907_lc_0907_sum_of_subarray_minimums_empty</t>
+          <t>lc_0907</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>monotonic_stack</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays;dynamic-programming</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>907 Lc 0907 Sum Of Subarray Minimums Empty</t>
+          <t>Sum of Subarray Minimums</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">

</xml_diff>

<commit_message>
Quick Update 2026-04-12 13:25
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
@@ -27,16 +27,61 @@
       <b val="1"/>
       <sz val="16"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F497D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F8FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,13 +89,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -448,1200 +528,1980 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="89.5703125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="17.85546875" customWidth="1" min="3" max="3"/>
-    <col width="41.28515625" customWidth="1" min="4" max="4"/>
-    <col width="39.85546875" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="10.42578125" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="41" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="50" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="48" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="12" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" customFormat="1" customHeight="1" s="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>path</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>difficulty</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>data_structures</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>my_impression</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>key_nugget</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>lc_0055</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays/055_lc_0055_jump_game.py</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>arrays</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>arrays;greedy;dynamic-programming</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Jump Game</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>greedy-scan</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="n"/>
+      <c r="L2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>lc_0152</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays/152_lc_152_maximum_product_subarray.py</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>arrays</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>arrays;dynamic-programming</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Maximum Product Subarray</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>dynamic-programming</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="n"/>
+      <c r="L3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>lc_0238</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays/238_lc_0238_product_of_array_except_self.py</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>arrays</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>arrays;prefix-sum;suffix-sum</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Product of Array Except Self</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>prefix-sum</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>lc_0462</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays/462_lc_0462_minimum_moves_to_equal_array_elements_ii.py</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>arrays</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>arrays;math;sorting;median</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Minimum Moves to Equal Array Elements II</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>sorting+median</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>lc_0001</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays_hashing/001_lc_0001_two_sum_empty.py</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>arrays_hashing</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>arrays_hashing;arrays;hash-table</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Two Sum</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>hashmap-lookup</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>hashmap</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>lc_0036</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays_hashing/036_lc_036_valid_sudoku_empty.py</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>arrays_hashing</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>arrays_hashing;hash-table;matrix;set</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Valid Sudoku</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>hashmap-validation</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>hashmap+array</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="n"/>
+      <c r="L7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>lc_0049</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays_hashing/049_lc_049_group_anagrams_empty.py</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>arrays_hashing</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>arrays_hashing;hash-table;strings;sorting</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Group Anagrams</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>hashmap-grouping</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>hashmap</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="n"/>
+      <c r="L8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>lc_0128</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays_hashing/128_lc_128_longest_consecutive_sequence_empty.py</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>arrays_hashing</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>arrays_hashing;hash-table;arrays;union-find</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Longest Consecutive Sequence</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>hashset-expansion</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>hashset</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="n"/>
+      <c r="L9" s="4" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>lc_0217</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays_hashing/217_lc_0217_contains_duplicate_empty.py</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>arrays_hashing</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>arrays_hashing;hash-table;arrays;sorting</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Contains Duplicate</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>hashset-dedup</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>hashset</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="n"/>
+      <c r="L10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>lc_0242</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays_hashing/242_lc_0242_valid_anagram_empty.py</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>arrays_hashing</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>arrays_hashing;hash-table;strings;sorting</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Valid Anagram</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>hashmap-counting</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>hashmap</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="n"/>
+      <c r="L11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>lc_0271</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays_hashing/271_lc_0271_encode_and_decode_strings_empty.py</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>arrays_hashing</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>arrays_hashing;strings;design;encoding</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Encode and Decode Strings</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>design-encode-decode</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>array+string</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="n"/>
+      <c r="L12" s="4" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>lc_0347</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays_hashing/347_lc_0347_top_k_frequent_elements_empty.py</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>arrays_hashing</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>arrays_hashing;hash-table;heap;bucket-sort;counting</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Top K Frequent Elements</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>bucket-sort</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>hashmap+bucket-array</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>lc_0560</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/arrays_hashing/560_lc_0560_subarray_sum_equals_k_empty.py</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>arrays_hashing</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>arrays_hashing;hash-table;prefix-sum;arrays</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Subarray Sum Equals K</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>prefix-sum+hashmap</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>hashmap</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>cs_drone_delivery_foot_distance</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>greedy</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>greedy;simulation;sorting</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Drone Delivery Foot Distance</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>codesignal</t>
         </is>
       </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="4" t="n"/>
+      <c r="L15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>cs_key_changes_counter</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>greedy</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>greedy;simulation;arrays;strings</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Key Changes Counter</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>codesignal</t>
         </is>
       </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr"/>
+      <c r="K16" s="4" t="n"/>
+      <c r="L16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>lc_custom_harmonious_buildings</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>greedy</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>greedy;math;array;sequence</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Harmonious Building Patterns</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>codesignal</t>
         </is>
       </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="4" t="n"/>
+      <c r="L17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>lc_custom_harmonious_buildings_flexible</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>greedy</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>greedy;math;median;geometry</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Harmonious Building Patterns (Flexible)</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>codesignal</t>
         </is>
       </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr"/>
+      <c r="K18" s="4" t="n"/>
+      <c r="L18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>lc_0042</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/monotonic_stack/042_lc_042_trapping_rain_water_empty.py</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>monotonic_stack</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>monotonic_stack;stack;monotonic-stack;two-pointers;dynamic-programming</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Trapping Rain Water</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>two-pointer</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="n"/>
+      <c r="L19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>lc_0084</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/monotonic_stack/084_lc_084_largest_rectangle_in_histogram_empty.py</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>monotonic_stack</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>monotonic-stack</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>stack+array</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>lc_0085</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/monotonic_stack/085_lc_085_maximal_rectangle_empty.py</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>monotonic_stack</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>monotonic_stack;stack;monotonic-stack;dynamic-programming;matrix</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Maximal Rectangle</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>monotonic-stack+dp</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>stack+array</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>lc_1019</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>monotonic_stack</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Next Greater Node In Linked List</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>monotonic-stack</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>stack+linked-list</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="n"/>
+      <c r="L22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>lc_1475</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>monotonic_stack</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>Final Prices With a Special Discount in a Shop</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>monotonic-stack</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="n"/>
+      <c r="L23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>lc_0907</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/monotonic_stack/907_lc_0907_sum_of_subarray_minimums_empty.py</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>monotonic_stack</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>monotonic_stack;stack;monotonic-stack;arrays;dynamic-programming</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Sum of Subarray Minimums</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>monotonic-stack+dp</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>stack+array</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="n"/>
+      <c r="L24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>cs_phone_battery_simulation</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>simulation</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>simulation;arrays</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>Phone Battery Simulation</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>codesignal</t>
         </is>
       </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr"/>
+      <c r="K25" s="4" t="n"/>
+      <c r="L25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>lc_0020</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>stack;string</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>Valid Parentheses</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>stack-matching</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="n"/>
+      <c r="L26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>lc_0496</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>Next Greater Element I</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>monotonic-stack</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>stack+hashmap</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="n"/>
+      <c r="L27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>lc_0000</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>Next Smaller Element</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr"/>
+      <c r="J28" s="3" t="inlineStr"/>
+      <c r="K28" s="4" t="n"/>
+      <c r="L28" s="4" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>lc_0084</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>monotonic-stack</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>stack+array</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="n"/>
+      <c r="L29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>lc_0853</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>Car Fleet</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>monotonic-stack+greedy</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>stack+array</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="n"/>
+      <c r="L30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>lc_0901</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>Online Stock Span</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>monotonic-stack</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="n"/>
+      <c r="L31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>lc_0150</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>stack;array;math</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>stack-evaluation</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="n"/>
+      <c r="L32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>lc_0239</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Sliding Window Maximum</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>monotonic-deque</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>deque</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="n"/>
+      <c r="L33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>lc_0496</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>Next Greater Element I</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>monotonic-stack</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>stack+hashmap</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="n"/>
+      <c r="L34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>lc_0503</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>stack;monotonic-stack;arrays;circular-array</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>Next Greater Element II</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>monotonic-stack</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>stack+array</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="n"/>
+      <c r="L35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>lc_0739</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>Daily Temperatures</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>monotonic-stack</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="n"/>
+      <c r="L36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>leetcode</t>
-        </is>
-      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>design-min-stack</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="n"/>
+      <c r="L37" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 13:39
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -1345,13 +1345,21 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="inlineStr"/>
-      <c r="J15" s="6" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>greedy-scan+sorting</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
       <c r="K15" s="4" t="n"/>
       <c r="L15" s="4" t="n"/>
     </row>
@@ -1386,18 +1394,26 @@
           <t>codesignal</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H16" s="7" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr"/>
-      <c r="J16" s="3" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>simulation</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="K16" s="4" t="n"/>
       <c r="L16" s="4" t="n"/>
     </row>
@@ -1442,8 +1458,16 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>greedy+math</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
       <c r="K17" s="4" t="n"/>
       <c r="L17" s="4" t="n"/>
     </row>
@@ -1488,8 +1512,16 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>greedy+math</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
       <c r="K18" s="4" t="n"/>
       <c r="L18" s="4" t="n"/>
     </row>
@@ -1853,13 +1885,21 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr"/>
-      <c r="J25" s="6" t="inlineStr"/>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>simulation</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>heap+deque</t>
+        </is>
+      </c>
       <c r="K25" s="4" t="n"/>
       <c r="L25" s="4" t="n"/>
     </row>
@@ -2007,13 +2047,21 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr"/>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>monotonic-stack</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
       <c r="K28" s="4" t="n"/>
       <c r="L28" s="4" t="n"/>
     </row>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 15:13
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1620" yWindow="5250" windowWidth="38700" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="index" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 18:11
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1620" yWindow="5250" windowWidth="38700" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="index" sheetId="1" state="visible" r:id="rId1"/>
@@ -30,7 +30,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -47,37 +47,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F497D"/>
+        <fgColor rgb="FF1F497D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F8FF"/>
+        <fgColor rgb="FFF2F8FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,17 +91,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -528,21 +529,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:L38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="41" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="50" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="80.44140625" bestFit="1" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="48" bestFit="1" customWidth="1" min="5" max="5"/>
     <col width="12" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="7" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="42" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="11" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" customFormat="1" customHeight="1" s="1">
@@ -610,12 +609,12 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>lc_0055</t>
+          <t>lc_0134</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays/055_lc_0055_jump_game.py</t>
+          <t>leetcode/by_topic/arrays/0134_lc_134_gas_station.py</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -625,12 +624,12 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>arrays;greedy;dynamic-programming</t>
+          <t>arrays;greedy</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Jump Game</t>
+          <t>Gas Station</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -664,12 +663,12 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>lc_0152</t>
+          <t>lc_0055</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays/152_lc_152_maximum_product_subarray.py</t>
+          <t>leetcode/by_topic/arrays/055_lc_0055_jump_game.py</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -679,12 +678,12 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>arrays;dynamic-programming</t>
+          <t>arrays;greedy;dynamic-programming</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Maximum Product Subarray</t>
+          <t>Jump Game</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -718,12 +717,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>lc_0238</t>
+          <t>lc_0152</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays/238_lc_0238_product_of_array_except_self.py</t>
+          <t>leetcode/by_topic/arrays/152_lc_152_maximum_product_subarray.py</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -733,12 +732,12 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>arrays;prefix-sum;suffix-sum</t>
+          <t>arrays;dynamic-programming</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Product of Array Except Self</t>
+          <t>Maximum Product Subarray</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -772,12 +771,12 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>lc_0462</t>
+          <t>lc_0238</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays/462_lc_0462_minimum_moves_to_equal_array_elements_ii.py</t>
+          <t>leetcode/by_topic/arrays/238_lc_0238_product_of_array_except_self.py</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -787,12 +786,12 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>arrays;math;sorting;median</t>
+          <t>arrays;prefix-sum;suffix-sum</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Minimum Moves to Equal Array Elements II</t>
+          <t>Product of Array Except Self</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -826,27 +825,27 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>lc_0001</t>
+          <t>lc_0462</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays_hashing/001_lc_0001_two_sum_empty.py</t>
+          <t>leetcode/by_topic/arrays/462_lc_0462_minimum_moves_to_equal_array_elements_ii.py</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>arrays_hashing</t>
+          <t>arrays</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>arrays_hashing;arrays;hash-table</t>
+          <t>arrays;math;sorting;median</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Two Sum</t>
+          <t>Minimum Moves to Equal Array Elements II</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -880,12 +879,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>lc_0036</t>
+          <t>lc_0001</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays_hashing/036_lc_036_valid_sudoku_empty.py</t>
+          <t>leetcode/by_topic/arrays_hashing/001_lc_0001_two_sum_empty.py</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -895,12 +894,12 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>arrays_hashing;hash-table;matrix;set</t>
+          <t>arrays_hashing;arrays;hash-table</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Valid Sudoku</t>
+          <t>Two Sum</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -934,12 +933,12 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>lc_0049</t>
+          <t>lc_0036</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays_hashing/049_lc_049_group_anagrams_empty.py</t>
+          <t>leetcode/by_topic/arrays_hashing/036_lc_036_valid_sudoku_empty.py</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -949,12 +948,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>arrays_hashing;hash-table;strings;sorting</t>
+          <t>arrays_hashing;hash-table;matrix;set</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Group Anagrams</t>
+          <t>Valid Sudoku</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -988,12 +987,12 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>lc_0128</t>
+          <t>lc_0049</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays_hashing/128_lc_128_longest_consecutive_sequence_empty.py</t>
+          <t>leetcode/by_topic/arrays_hashing/049_lc_049_group_anagrams_empty.py</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1003,12 +1002,12 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>arrays_hashing;hash-table;arrays;union-find</t>
+          <t>arrays_hashing;hash-table;strings;sorting</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Longest Consecutive Sequence</t>
+          <t>Group Anagrams</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -1042,12 +1041,12 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>lc_0217</t>
+          <t>lc_0128</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays_hashing/217_lc_0217_contains_duplicate_empty.py</t>
+          <t>leetcode/by_topic/arrays_hashing/128_lc_128_longest_consecutive_sequence_empty.py</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1057,12 +1056,12 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>arrays_hashing;hash-table;arrays;sorting</t>
+          <t>arrays_hashing;hash-table;arrays;union-find</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Contains Duplicate</t>
+          <t>Longest Consecutive Sequence</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1096,12 +1095,12 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>lc_0242</t>
+          <t>lc_0217</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays_hashing/242_lc_0242_valid_anagram_empty.py</t>
+          <t>leetcode/by_topic/arrays_hashing/217_lc_0217_contains_duplicate_empty.py</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1111,12 +1110,12 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>arrays_hashing;hash-table;strings;sorting</t>
+          <t>arrays_hashing;hash-table;arrays;sorting</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Valid Anagram</t>
+          <t>Contains Duplicate</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1150,12 +1149,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>lc_0271</t>
+          <t>lc_0242</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays_hashing/271_lc_0271_encode_and_decode_strings_empty.py</t>
+          <t>leetcode/by_topic/arrays_hashing/242_lc_0242_valid_anagram_empty.py</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1165,12 +1164,12 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>arrays_hashing;strings;design;encoding</t>
+          <t>arrays_hashing;hash-table;strings;sorting</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Encode and Decode Strings</t>
+          <t>Valid Anagram</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1204,12 +1203,12 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>lc_0347</t>
+          <t>lc_0271</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays_hashing/347_lc_0347_top_k_frequent_elements_empty.py</t>
+          <t>leetcode/by_topic/arrays_hashing/271_lc_0271_encode_and_decode_strings_empty.py</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1219,12 +1218,12 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>arrays_hashing;hash-table;heap;bucket-sort;counting</t>
+          <t>arrays_hashing;strings;design;encoding</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Top K Frequent Elements</t>
+          <t>Encode and Decode Strings</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1258,12 +1257,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>lc_0560</t>
+          <t>lc_0347</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/arrays_hashing/560_lc_0560_subarray_sum_equals_k_empty.py</t>
+          <t>leetcode/by_topic/arrays_hashing/347_lc_0347_top_k_frequent_elements_empty.py</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1273,12 +1272,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>arrays_hashing;hash-table;prefix-sum;arrays</t>
+          <t>arrays_hashing;hash-table;heap;bucket-sort;counting</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Subarray Sum Equals K</t>
+          <t>Top K Frequent Elements</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1312,32 +1311,32 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>cs_drone_delivery_foot_distance</t>
+          <t>lc_0560</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
+          <t>leetcode/by_topic/arrays_hashing/560_lc_0560_subarray_sum_equals_k_empty.py</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>greedy</t>
+          <t>arrays_hashing</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>greedy;simulation;sorting</t>
+          <t>arrays_hashing;hash-table;prefix-sum;arrays</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Drone Delivery Foot Distance</t>
+          <t>Subarray Sum Equals K</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1366,12 +1365,12 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>cs_key_changes_counter</t>
+          <t>cs_drone_delivery_foot_distance</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
+          <t>leetcode/by_topic/greedy/cs_drone_delivery_foot_distance.py</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1381,12 +1380,12 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>greedy;simulation;arrays;strings</t>
+          <t>greedy;simulation;sorting</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Key Changes Counter</t>
+          <t>Drone Delivery Foot Distance</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1420,12 +1419,12 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings</t>
+          <t>cs_key_changes_counter</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
+          <t>leetcode/by_topic/greedy/cs_key_changes_counter.py</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -1435,12 +1434,12 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>greedy;math;array;sequence</t>
+          <t>greedy;simulation;arrays;strings</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns</t>
+          <t>Key Changes Counter</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1474,12 +1473,12 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>lc_custom_harmonious_buildings_flexible</t>
+          <t>lc_custom_harmonious_buildings</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
+          <t>leetcode/by_topic/greedy/custom_codesignal_harmonious_building_patterns.py</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1489,12 +1488,12 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>greedy;math;median;geometry</t>
+          <t>greedy;math;array;sequence</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Harmonious Building Patterns (Flexible)</t>
+          <t>Harmonious Building Patterns</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1528,32 +1527,32 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>lc_0042</t>
+          <t>lc_custom_harmonious_buildings_flexible</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/042_lc_042_trapping_rain_water_empty.py</t>
+          <t>leetcode/by_topic/greedy/custom_harmonious_building_patterns_flexible.py</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>monotonic_stack</t>
+          <t>greedy</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;two-pointers;dynamic-programming</t>
+          <t>greedy;math;median;geometry</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Trapping Rain Water</t>
+          <t>Harmonious Building Patterns (Flexible)</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -1582,12 +1581,12 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0042</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/084_lc_084_largest_rectangle_in_histogram_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/042_lc_042_trapping_rain_water_empty.py</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1597,12 +1596,12 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;two-pointers;dynamic-programming</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Trapping Rain Water</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1636,12 +1635,12 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>lc_0085</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/085_lc_085_maximal_rectangle_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/084_lc_084_largest_rectangle_in_histogram_empty.py</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -1651,12 +1650,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;dynamic-programming;matrix</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Maximal Rectangle</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1690,12 +1689,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>lc_1019</t>
+          <t>lc_0085</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/085_lc_085_maximal_rectangle_empty.py</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1705,12 +1704,12 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;dynamic-programming;matrix</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Next Greater Node In Linked List</t>
+          <t>Maximal Rectangle</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1744,12 +1743,12 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>lc_1475</t>
+          <t>lc_1019</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -1759,12 +1758,12 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Final Prices With a Special Discount in a Shop</t>
+          <t>Next Greater Node In Linked List</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1798,12 +1797,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>lc_0907</t>
+          <t>lc_1475</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/907_lc_0907_sum_of_subarray_minimums_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1813,12 +1812,12 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;arrays;dynamic-programming</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Sum of Subarray Minimums</t>
+          <t>Final Prices With a Special Discount in a Shop</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1846,38 +1845,42 @@
           <t>stack+array</t>
         </is>
       </c>
-      <c r="K24" s="4" t="n"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Very difficult. I do not even Know how to start it!!!</t>
+        </is>
+      </c>
       <c r="L24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_0907</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/monotonic_stack/907_lc_0907_sum_of_subarray_minimums_empty.py</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>monotonic_stack</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays;dynamic-programming</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Sum of Subarray Minimums</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1906,32 +1909,32 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1960,12 +1963,12 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1975,12 +1978,12 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -2014,12 +2017,12 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -2034,7 +2037,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -2068,12 +2071,12 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -2088,7 +2091,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -2122,12 +2125,12 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2137,12 +2140,12 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -2176,12 +2179,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -2191,12 +2194,12 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -2230,12 +2233,12 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2245,12 +2248,12 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -2284,12 +2287,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -2299,12 +2302,12 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -2338,12 +2341,12 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2353,12 +2356,12 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -2392,12 +2395,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -2407,12 +2410,12 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -2446,12 +2449,12 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0503</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2461,12 +2464,12 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element II</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -2500,12 +2503,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>lc_0155</t>
+          <t>lc_0739</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -2515,12 +2518,12 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>stack;design</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Min Stack</t>
+          <t>Daily Temperatures</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -2550,6 +2553,38 @@
       </c>
       <c r="K37" s="4" t="n"/>
       <c r="L37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>lc_0155</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>stack;design</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Min Stack</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 19:31
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="41" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1581,27 +1581,27 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>lc_0042</t>
+          <t>047_lc_2532_time_to_cross_a_bridge_empty</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/042_lc_042_trapping_rain_water_empty.py</t>
+          <t>leetcode/by_topic/heap_priority_queue/047_lc_2532_time_to_cross_a_bridge_empty.py</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>monotonic_stack</t>
+          <t>heap_priority_queue</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;two-pointers;dynamic-programming</t>
+          <t>heap_priority_queue</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Trapping Rain Water</t>
+          <t>047 Lc 2532 Time To Cross A Bridge Empty</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1635,12 +1635,12 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0042</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/084_lc_084_largest_rectangle_in_histogram_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/042_lc_042_trapping_rain_water_empty.py</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -1650,12 +1650,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;two-pointers;dynamic-programming</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Trapping Rain Water</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1689,12 +1689,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>lc_0085</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/085_lc_085_maximal_rectangle_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/084_lc_084_largest_rectangle_in_histogram_empty.py</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1704,12 +1704,12 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;dynamic-programming;matrix</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Maximal Rectangle</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1743,12 +1743,12 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>lc_1019</t>
+          <t>lc_0085</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/085_lc_085_maximal_rectangle_empty.py</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -1758,12 +1758,12 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;dynamic-programming;matrix</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Next Greater Node In Linked List</t>
+          <t>Maximal Rectangle</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1797,12 +1797,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>lc_1475</t>
+          <t>lc_1019</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1019_lc_1019_next_greater_node_in_linked_list_empty.py</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1812,12 +1812,12 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
+          <t>monotonic_stack;linked-list;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Final Prices With a Special Discount in a Shop</t>
+          <t>Next Greater Node In Linked List</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1855,12 +1855,12 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>lc_0907</t>
+          <t>lc_1475</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/monotonic_stack/907_lc_0907_sum_of_subarray_minimums_empty.py</t>
+          <t>leetcode/by_topic/monotonic_stack/1475_lc_1475_final_prices_with_special_discount_empty.py</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -1870,12 +1870,12 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>monotonic_stack;stack;monotonic-stack;arrays;dynamic-programming</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Sum of Subarray Minimums</t>
+          <t>Final Prices With a Special Discount in a Shop</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -1909,32 +1909,32 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>cs_phone_battery_simulation</t>
+          <t>lc_0907</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
+          <t>leetcode/by_topic/monotonic_stack/907_lc_0907_sum_of_subarray_minimums_empty.py</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>simulation</t>
+          <t>monotonic_stack</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>simulation;arrays</t>
+          <t>monotonic_stack;stack;monotonic-stack;arrays;dynamic-programming</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Phone Battery Simulation</t>
+          <t>Sum of Subarray Minimums</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>codesignal</t>
+          <t>leetcode</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1963,32 +1963,32 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>lc_0020</t>
+          <t>cs_phone_battery_simulation</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
+          <t>leetcode/by_topic/simulation/cs_phone_battery_simulation.py</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>stack</t>
+          <t>simulation</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>stack;string</t>
+          <t>simulation;arrays</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Phone Battery Simulation</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>leetcode</t>
+          <t>codesignal</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -2017,12 +2017,12 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0020</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/020_lc_0020_valid_parentheses.py</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -2032,12 +2032,12 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;string</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Valid Parentheses</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -2071,12 +2071,12 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>lc_0000</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
+          <t>leetcode/by_topic/stack/024_next_greater_single_list_empty.py</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Next Smaller Element</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -2125,12 +2125,12 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>lc_0084</t>
+          <t>lc_0000</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
+          <t>leetcode/by_topic/stack/025_next_smaller_single_list_empty.py</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Largest Rectangle in Histogram</t>
+          <t>Next Smaller Element</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -2179,12 +2179,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>lc_0853</t>
+          <t>lc_0084</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
+          <t>leetcode/by_topic/stack/084_lc_0084_largest_rectangle_in_histogram.py</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -2194,12 +2194,12 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>stack;greedy;sorting;arrays</t>
+          <t>stack;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Car Fleet</t>
+          <t>Largest Rectangle in Histogram</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -2233,12 +2233,12 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>lc_0901</t>
+          <t>lc_0853</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
+          <t>leetcode/by_topic/stack/0853_lc_0853_car_fleet_empty.py</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2248,12 +2248,12 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>stack;design;monotonic-stack;data-stream</t>
+          <t>stack;greedy;sorting;arrays</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Online Stock Span</t>
+          <t>Car Fleet</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -2287,12 +2287,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>lc_0150</t>
+          <t>lc_0901</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
+          <t>leetcode/by_topic/stack/0901_lc_901_online_stock_span.py</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -2302,12 +2302,12 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>stack;array;math</t>
+          <t>stack;design;monotonic-stack;data-stream</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Online Stock Span</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -2341,12 +2341,12 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>lc_0239</t>
+          <t>lc_0150</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
+          <t>leetcode/by_topic/stack/150_lc_0150_evaluate_reverse_polish_notation.py</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2356,12 +2356,12 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
+          <t>stack;array;math</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Sliding Window Maximum</t>
+          <t>Evaluate Reverse Polish Notation</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -2395,12 +2395,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>lc_0496</t>
+          <t>lc_0239</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
+          <t>leetcode/by_topic/stack/239_lc_0239_sliding_window_maximum.py</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -2410,12 +2410,12 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>stack;hash-table;monotonic-stack;arrays</t>
+          <t>stack;sliding-window;heap;queue;monotonic-queue</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Sliding Window Maximum</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -2449,12 +2449,12 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>lc_0503</t>
+          <t>lc_0496</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
+          <t>leetcode/by_topic/stack/496_lc_0496_next_greater_element_i_empty.py</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays;circular-array</t>
+          <t>stack;hash-table;monotonic-stack;arrays</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Next Greater Element II</t>
+          <t>Next Greater Element I</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -2503,12 +2503,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>lc_0739</t>
+          <t>lc_0503</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+          <t>leetcode/by_topic/stack/503_lc_0503_next_greater_element_ii_empty.py</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -2518,12 +2518,12 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>stack;monotonic-stack;arrays</t>
+          <t>stack;monotonic-stack;arrays;circular-array</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Next Greater Element II</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -2557,30 +2557,62 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
+          <t>lc_0739</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>leetcode/by_topic/stack/739_lc_0739_daily_temperatures_empty.py</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>stack</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>stack;monotonic-stack;arrays</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>leetcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
           <t>lc_0155</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>leetcode/by_topic/stack/lc_0155_min_stack.py</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>stack</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>stack;design</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Min Stack</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>leetcode</t>
         </is>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 21:15
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="index" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 21:40
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="index" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Quick Update 2026-04-12 22:45
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="index" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Quick Update 2026-04-13 14:42
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="index" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Quick Update 2026-04-13 15:56
# Conflicts:
#	coding_challenges/index.xlsx
</commit_message>
<xml_diff>
--- a/coding_challenges/index.xlsx
+++ b/coding_challenges/index.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="index" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>

</xml_diff>